<commit_message>
add pitch video link to project documentation
</commit_message>
<xml_diff>
--- a/docs/Projektfeladat8.xlsx
+++ b/docs/Projektfeladat8.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\webprog_alapjai_d5qd9q\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81F42634-AC9A-4D70-A8C9-AF92F03EEFD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF360E96-0B19-4262-9056-727D6C7CBEFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4275" yWindow="1155" windowWidth="24330" windowHeight="14895" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6030" yWindow="1290" windowWidth="29055" windowHeight="17985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Munka1" sheetId="1" r:id="rId1"/>
@@ -1078,22 +1078,16 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1105,13 +1099,40 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1123,44 +1144,23 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1391,7 +1391,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="10"/>
@@ -1421,7 +1421,7 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="34" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
@@ -1495,16 +1495,16 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="17"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="15"/>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
@@ -1527,14 +1527,14 @@
       <c r="Z4" s="1"/>
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="14"/>
-      <c r="B5" s="18" t="s">
+      <c r="A5" s="21"/>
+      <c r="B5" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="20"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="24"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -1558,11 +1558,11 @@
     </row>
     <row r="6" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="12"/>
-      <c r="B6" s="21"/>
+      <c r="B6" s="28"/>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
-      <c r="F6" s="22"/>
+      <c r="F6" s="29"/>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
@@ -1585,16 +1585,16 @@
       <c r="Z6" s="1"/>
     </row>
     <row r="7" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="17"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="15"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
@@ -1617,14 +1617,14 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14"/>
-      <c r="B8" s="24" t="s">
+      <c r="A8" s="21"/>
+      <c r="B8" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="17"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="15"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
@@ -1647,16 +1647,16 @@
       <c r="Z8" s="1"/>
     </row>
     <row r="9" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="14"/>
+      <c r="A9" s="21"/>
       <c r="B9" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="30" t="s">
         <v>15</v>
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
-      <c r="F9" s="22"/>
+      <c r="F9" s="29"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
@@ -1679,16 +1679,16 @@
       <c r="Z9" s="1"/>
     </row>
     <row r="10" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="14"/>
+      <c r="A10" s="21"/>
       <c r="B10" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="23" t="s">
+      <c r="C10" s="30" t="s">
         <v>15</v>
       </c>
       <c r="D10" s="10"/>
       <c r="E10" s="10"/>
-      <c r="F10" s="22"/>
+      <c r="F10" s="29"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -1711,16 +1711,16 @@
       <c r="Z10" s="1"/>
     </row>
     <row r="11" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14"/>
+      <c r="A11" s="21"/>
       <c r="B11" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="30" t="s">
         <v>15</v>
       </c>
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
-      <c r="F11" s="22"/>
+      <c r="F11" s="29"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
@@ -1743,16 +1743,16 @@
       <c r="Z11" s="1"/>
     </row>
     <row r="12" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="14"/>
+      <c r="A12" s="21"/>
       <c r="B12" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="23" t="s">
+      <c r="C12" s="30" t="s">
         <v>15</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="10"/>
-      <c r="F12" s="22"/>
+      <c r="F12" s="29"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -1775,16 +1775,16 @@
       <c r="Z12" s="1"/>
     </row>
     <row r="13" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="14"/>
+      <c r="A13" s="21"/>
       <c r="B13" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="30" t="s">
         <v>15</v>
       </c>
       <c r="D13" s="10"/>
       <c r="E13" s="10"/>
-      <c r="F13" s="22"/>
+      <c r="F13" s="29"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
@@ -1807,16 +1807,16 @@
       <c r="Z13" s="1"/>
     </row>
     <row r="14" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="14"/>
+      <c r="A14" s="21"/>
       <c r="B14" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="23" t="s">
+      <c r="C14" s="30" t="s">
         <v>15</v>
       </c>
       <c r="D14" s="10"/>
       <c r="E14" s="10"/>
-      <c r="F14" s="22"/>
+      <c r="F14" s="29"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
@@ -1839,16 +1839,16 @@
       <c r="Z14" s="1"/>
     </row>
     <row r="15" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="14"/>
+      <c r="A15" s="21"/>
       <c r="B15" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="C15" s="30" t="s">
         <v>15</v>
       </c>
       <c r="D15" s="10"/>
       <c r="E15" s="10"/>
-      <c r="F15" s="22"/>
+      <c r="F15" s="29"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
@@ -1871,16 +1871,16 @@
       <c r="Z15" s="1"/>
     </row>
     <row r="16" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="14"/>
+      <c r="A16" s="21"/>
       <c r="B16" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="C16" s="30" t="s">
         <v>15</v>
       </c>
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
-      <c r="F16" s="22"/>
+      <c r="F16" s="29"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
@@ -1903,16 +1903,16 @@
       <c r="Z16" s="1"/>
     </row>
     <row r="17" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="14"/>
+      <c r="A17" s="21"/>
       <c r="B17" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="30" t="s">
         <v>15</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
-      <c r="F17" s="22"/>
+      <c r="F17" s="29"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
@@ -1935,16 +1935,16 @@
       <c r="Z17" s="1"/>
     </row>
     <row r="18" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="14"/>
+      <c r="A18" s="21"/>
       <c r="B18" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="23" t="s">
+      <c r="C18" s="30" t="s">
         <v>15</v>
       </c>
       <c r="D18" s="10"/>
       <c r="E18" s="10"/>
-      <c r="F18" s="22"/>
+      <c r="F18" s="29"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
@@ -1967,16 +1967,16 @@
       <c r="Z18" s="1"/>
     </row>
     <row r="19" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="14"/>
+      <c r="A19" s="21"/>
       <c r="B19" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="30" t="s">
         <v>15</v>
       </c>
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
-      <c r="F19" s="22"/>
+      <c r="F19" s="29"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
@@ -2003,12 +2003,12 @@
       <c r="B20" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="23" t="s">
+      <c r="C20" s="30" t="s">
         <v>15</v>
       </c>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
-      <c r="F20" s="22"/>
+      <c r="F20" s="29"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -2031,16 +2031,16 @@
       <c r="Z20" s="1"/>
     </row>
     <row r="21" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
+      <c r="A21" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="15" t="s">
+      <c r="B21" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="17"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="15"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
@@ -2064,13 +2064,13 @@
     </row>
     <row r="22" spans="1:26" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="12"/>
-      <c r="B22" s="35" t="s">
+      <c r="B22" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="17"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="15"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
@@ -2093,16 +2093,16 @@
       <c r="Z22" s="1"/>
     </row>
     <row r="23" spans="1:26" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="15" t="s">
+      <c r="B23" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="16"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="17"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="15"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
@@ -2126,13 +2126,13 @@
     </row>
     <row r="24" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="12"/>
-      <c r="B24" s="36" t="s">
+      <c r="B24" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="17"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="15"/>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
@@ -2155,16 +2155,16 @@
       <c r="Z24" s="1"/>
     </row>
     <row r="25" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B25" s="15" t="s">
+      <c r="B25" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="17"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="15"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
@@ -2188,13 +2188,13 @@
     </row>
     <row r="26" spans="1:26" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="10"/>
-      <c r="B26" s="26" t="s">
+      <c r="B26" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="17"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="15"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
@@ -2217,16 +2217,16 @@
       <c r="Z26" s="1"/>
     </row>
     <row r="27" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="28" t="s">
+      <c r="A27" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B27" s="29" t="s">
+      <c r="B27" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="17"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="15"/>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
@@ -2250,13 +2250,13 @@
     </row>
     <row r="28" spans="1:26" ht="173.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="10"/>
-      <c r="B28" s="30" t="s">
+      <c r="B28" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="17"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="15"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
@@ -2279,16 +2279,16 @@
       <c r="Z28" s="1"/>
     </row>
     <row r="29" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B29" s="29" t="s">
+      <c r="B29" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="17"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="15"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
@@ -2311,14 +2311,14 @@
       <c r="Z29" s="1"/>
     </row>
     <row r="30" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="14"/>
-      <c r="B30" s="31" t="s">
+      <c r="A30" s="21"/>
+      <c r="B30" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="20"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="23"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="24"/>
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
@@ -2341,12 +2341,12 @@
       <c r="Z30" s="1"/>
     </row>
     <row r="31" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="14"/>
-      <c r="B31" s="32"/>
-      <c r="C31" s="33"/>
-      <c r="D31" s="33"/>
-      <c r="E31" s="33"/>
-      <c r="F31" s="34"/>
+      <c r="A31" s="21"/>
+      <c r="B31" s="25"/>
+      <c r="C31" s="26"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="27"/>
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
@@ -2369,12 +2369,12 @@
       <c r="Z31" s="1"/>
     </row>
     <row r="32" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="14"/>
-      <c r="B32" s="32"/>
-      <c r="C32" s="33"/>
-      <c r="D32" s="33"/>
-      <c r="E32" s="33"/>
-      <c r="F32" s="34"/>
+      <c r="A32" s="21"/>
+      <c r="B32" s="25"/>
+      <c r="C32" s="26"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="27"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
@@ -2397,12 +2397,12 @@
       <c r="Z32" s="1"/>
     </row>
     <row r="33" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="14"/>
-      <c r="B33" s="32"/>
-      <c r="C33" s="33"/>
-      <c r="D33" s="33"/>
-      <c r="E33" s="33"/>
-      <c r="F33" s="34"/>
+      <c r="A33" s="21"/>
+      <c r="B33" s="25"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="26"/>
+      <c r="F33" s="27"/>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
@@ -2425,12 +2425,12 @@
       <c r="Z33" s="1"/>
     </row>
     <row r="34" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="14"/>
-      <c r="B34" s="32"/>
-      <c r="C34" s="33"/>
-      <c r="D34" s="33"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="34"/>
+      <c r="A34" s="21"/>
+      <c r="B34" s="25"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="26"/>
+      <c r="F34" s="27"/>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
@@ -2453,12 +2453,12 @@
       <c r="Z34" s="1"/>
     </row>
     <row r="35" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="14"/>
-      <c r="B35" s="32"/>
-      <c r="C35" s="33"/>
-      <c r="D35" s="33"/>
-      <c r="E35" s="33"/>
-      <c r="F35" s="34"/>
+      <c r="A35" s="21"/>
+      <c r="B35" s="25"/>
+      <c r="C35" s="26"/>
+      <c r="D35" s="26"/>
+      <c r="E35" s="26"/>
+      <c r="F35" s="27"/>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
@@ -2481,12 +2481,12 @@
       <c r="Z35" s="1"/>
     </row>
     <row r="36" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="14"/>
-      <c r="B36" s="32"/>
-      <c r="C36" s="33"/>
-      <c r="D36" s="33"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="34"/>
+      <c r="A36" s="21"/>
+      <c r="B36" s="25"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="26"/>
+      <c r="E36" s="26"/>
+      <c r="F36" s="27"/>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
@@ -2509,12 +2509,12 @@
       <c r="Z36" s="1"/>
     </row>
     <row r="37" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="14"/>
-      <c r="B37" s="32"/>
-      <c r="C37" s="33"/>
-      <c r="D37" s="33"/>
-      <c r="E37" s="33"/>
-      <c r="F37" s="34"/>
+      <c r="A37" s="21"/>
+      <c r="B37" s="25"/>
+      <c r="C37" s="26"/>
+      <c r="D37" s="26"/>
+      <c r="E37" s="26"/>
+      <c r="F37" s="27"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
@@ -2537,12 +2537,12 @@
       <c r="Z37" s="1"/>
     </row>
     <row r="38" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="14"/>
-      <c r="B38" s="32"/>
-      <c r="C38" s="33"/>
-      <c r="D38" s="33"/>
-      <c r="E38" s="33"/>
-      <c r="F38" s="34"/>
+      <c r="A38" s="21"/>
+      <c r="B38" s="25"/>
+      <c r="C38" s="26"/>
+      <c r="D38" s="26"/>
+      <c r="E38" s="26"/>
+      <c r="F38" s="27"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
@@ -2565,12 +2565,12 @@
       <c r="Z38" s="1"/>
     </row>
     <row r="39" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="14"/>
-      <c r="B39" s="32"/>
-      <c r="C39" s="33"/>
-      <c r="D39" s="33"/>
-      <c r="E39" s="33"/>
-      <c r="F39" s="34"/>
+      <c r="A39" s="21"/>
+      <c r="B39" s="25"/>
+      <c r="C39" s="26"/>
+      <c r="D39" s="26"/>
+      <c r="E39" s="26"/>
+      <c r="F39" s="27"/>
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
@@ -2593,12 +2593,12 @@
       <c r="Z39" s="1"/>
     </row>
     <row r="40" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="14"/>
-      <c r="B40" s="32"/>
-      <c r="C40" s="33"/>
-      <c r="D40" s="33"/>
-      <c r="E40" s="33"/>
-      <c r="F40" s="34"/>
+      <c r="A40" s="21"/>
+      <c r="B40" s="25"/>
+      <c r="C40" s="26"/>
+      <c r="D40" s="26"/>
+      <c r="E40" s="26"/>
+      <c r="F40" s="27"/>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
@@ -2622,11 +2622,11 @@
     </row>
     <row r="41" spans="1:26" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="12"/>
-      <c r="B41" s="21"/>
+      <c r="B41" s="28"/>
       <c r="C41" s="10"/>
       <c r="D41" s="10"/>
       <c r="E41" s="10"/>
-      <c r="F41" s="22"/>
+      <c r="F41" s="29"/>
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
@@ -2649,16 +2649,16 @@
       <c r="Z41" s="1"/>
     </row>
     <row r="42" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="13" t="s">
+      <c r="A42" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B42" s="25" t="s">
+      <c r="B42" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="C42" s="16"/>
-      <c r="D42" s="16"/>
-      <c r="E42" s="16"/>
-      <c r="F42" s="17"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="15"/>
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
@@ -2682,13 +2682,13 @@
     </row>
     <row r="43" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="12"/>
-      <c r="B43" s="27" t="s">
+      <c r="B43" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="C43" s="16"/>
-      <c r="D43" s="16"/>
-      <c r="E43" s="16"/>
-      <c r="F43" s="17"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="15"/>
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
@@ -29368,28 +29368,6 @@
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B22:F22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="B23:F23"/>
-    <mergeCell ref="B24:F24"/>
-    <mergeCell ref="B43:F43"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="A29:A41"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B30:F41"/>
-    <mergeCell ref="A42:A43"/>
-    <mergeCell ref="C10:F10"/>
-    <mergeCell ref="C11:F11"/>
-    <mergeCell ref="C12:F12"/>
-    <mergeCell ref="B42:F42"/>
-    <mergeCell ref="B25:F25"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="C19:F19"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="A4:A6"/>
@@ -29406,6 +29384,28 @@
     <mergeCell ref="C17:F17"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="C9:F9"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="C11:F11"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="B42:F42"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="C19:F19"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="A29:A41"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B30:F41"/>
+    <mergeCell ref="A42:A43"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B24:F24"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F3" r:id="rId1" xr:uid="{A7B8E26E-FC4C-4AF1-8A50-0EBA09BECB97}"/>
@@ -29416,14 +29416,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f5a9b5a3-46da-4859-9184-5bd2a5992ed5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="e80db319-43ef-461c-99bf-8c5167bc175f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -29628,21 +29626,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f5a9b5a3-46da-4859-9184-5bd2a5992ed5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="e80db319-43ef-461c-99bf-8c5167bc175f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26A1B02F-C0E5-4884-B3F9-F8FFA81F3B24}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D84E25B1-2683-4851-922F-A21F6B1F8698}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f5a9b5a3-46da-4859-9184-5bd2a5992ed5"/>
-    <ds:schemaRef ds:uri="e80db319-43ef-461c-99bf-8c5167bc175f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -29667,9 +29664,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D84E25B1-2683-4851-922F-A21F6B1F8698}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26A1B02F-C0E5-4884-B3F9-F8FFA81F3B24}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f5a9b5a3-46da-4859-9184-5bd2a5992ed5"/>
+    <ds:schemaRef ds:uri="e80db319-43ef-461c-99bf-8c5167bc175f"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>